<commit_message>
Add licenses (CC BY 4.0 for data, MIT for code) and correct the workbook version stamp
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CESBench-EN-v20260902.xlsx
+++ b/CESBench-EN-v20260902.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>v20260807</t>
+          <t>v20260902</t>
         </is>
       </c>
     </row>
@@ -582,6 +582,7 @@
         <v>370</v>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -775,6 +776,7 @@
         <v>370</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>

</xml_diff>